<commit_message>
Added names of countries and updated flag status
</commit_message>
<xml_diff>
--- a/countries_progress.xlsx
+++ b/countries_progress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Desktop\Modern-Day-Mod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E529B34-2025-4632-8366-16859DF5A235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE84AA3-5827-4FFF-B8F6-6B3DE038D532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15540" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
+    <workbookView xWindow="25200" yWindow="0" windowWidth="12600" windowHeight="15300" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="407">
   <si>
     <t>SWI</t>
   </si>
@@ -684,6 +684,579 @@
   </si>
   <si>
     <t>Langugaes</t>
+  </si>
+  <si>
+    <t>Angola</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Armenia</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Azerbaijan</t>
+  </si>
+  <si>
+    <t>Bahamas</t>
+  </si>
+  <si>
+    <t>Bahrain</t>
+  </si>
+  <si>
+    <t>Bangladesh</t>
+  </si>
+  <si>
+    <t>Barbados</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>Belarus</t>
+  </si>
+  <si>
+    <t>Belize</t>
+  </si>
+  <si>
+    <t>Benin</t>
+  </si>
+  <si>
+    <t>Bhutan</t>
+  </si>
+  <si>
+    <t>Bolivia</t>
+  </si>
+  <si>
+    <t>Antigua and Barbuda</t>
+  </si>
+  <si>
+    <t>Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>Brunei</t>
+  </si>
+  <si>
+    <t>Andorra</t>
+  </si>
+  <si>
+    <t>Botswana</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Burkina Faso</t>
+  </si>
+  <si>
+    <t>Bulgaria</t>
+  </si>
+  <si>
+    <t>Burundi</t>
+  </si>
+  <si>
+    <t>Central African Republic</t>
+  </si>
+  <si>
+    <t>Cameroon</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Chad</t>
+  </si>
+  <si>
+    <t>Chechnya</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t>Congo</t>
+  </si>
+  <si>
+    <t>Comoros</t>
+  </si>
+  <si>
+    <t>Costa Rica</t>
+  </si>
+  <si>
+    <t>Cabo Verde</t>
+  </si>
+  <si>
+    <t>Croatia</t>
+  </si>
+  <si>
+    <t>Cuba</t>
+  </si>
+  <si>
+    <t>Cyprus</t>
+  </si>
+  <si>
+    <t>Czech Republic</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Maldives</t>
+  </si>
+  <si>
+    <t>Djibouti</t>
+  </si>
+  <si>
+    <t>Dominica</t>
+  </si>
+  <si>
+    <t>Democratic Republic of the Congo</t>
+  </si>
+  <si>
+    <t>Ecuador</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>El Salvador</t>
+  </si>
+  <si>
+    <t>Equatorial Guinea</t>
+  </si>
+  <si>
+    <t>Eritrea</t>
+  </si>
+  <si>
+    <t>Estonia</t>
+  </si>
+  <si>
+    <t>Eswatini</t>
+  </si>
+  <si>
+    <t>Ethiopia</t>
+  </si>
+  <si>
+    <t>Timor-Leste</t>
+  </si>
+  <si>
+    <t>Fiji</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Gabon</t>
+  </si>
+  <si>
+    <t>Gambia</t>
+  </si>
+  <si>
+    <t>Guinea-Bissau</t>
+  </si>
+  <si>
+    <t>Great Britain</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Ghana</t>
+  </si>
+  <si>
+    <t>Greece</t>
+  </si>
+  <si>
+    <t>Grenada</t>
+  </si>
+  <si>
+    <t>Guatemala</t>
+  </si>
+  <si>
+    <t>Guinea</t>
+  </si>
+  <si>
+    <t>Guyana</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Haiti</t>
+  </si>
+  <si>
+    <t>Honduras</t>
+  </si>
+  <si>
+    <t>Hungary</t>
+  </si>
+  <si>
+    <t>Iceland</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t>Iran</t>
+  </si>
+  <si>
+    <t>Iraq</t>
+  </si>
+  <si>
+    <t>Ireland</t>
+  </si>
+  <si>
+    <t>Israel</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Côte d'Ivoire</t>
+  </si>
+  <si>
+    <t>Jamaica</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Kazakhstan</t>
+  </si>
+  <si>
+    <t>Kenya</t>
+  </si>
+  <si>
+    <t>Cambodia</t>
+  </si>
+  <si>
+    <t>Kiribati</t>
+  </si>
+  <si>
+    <t>Kosovo</t>
+  </si>
+  <si>
+    <t>Kuwait</t>
+  </si>
+  <si>
+    <t>Kyrgyzstan</t>
+  </si>
+  <si>
+    <t>Laos</t>
+  </si>
+  <si>
+    <t>Latvia</t>
+  </si>
+  <si>
+    <t>Lebanon</t>
+  </si>
+  <si>
+    <t>Lesotho</t>
+  </si>
+  <si>
+    <t>Liberia</t>
+  </si>
+  <si>
+    <t>Libya</t>
+  </si>
+  <si>
+    <t>Lithuania</t>
+  </si>
+  <si>
+    <t>Luxembourg</t>
+  </si>
+  <si>
+    <t>Madagascar</t>
+  </si>
+  <si>
+    <t>North Macedonia</t>
+  </si>
+  <si>
+    <t>Mali</t>
+  </si>
+  <si>
+    <t>Malaysia</t>
+  </si>
+  <si>
+    <t>Malta</t>
+  </si>
+  <si>
+    <t>Malawi</t>
+  </si>
+  <si>
+    <t>Marshall Islands</t>
+  </si>
+  <si>
+    <t>Mauritius</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>Mongolia</t>
+  </si>
+  <si>
+    <t>Moldova</t>
+  </si>
+  <si>
+    <t>Micronesia</t>
+  </si>
+  <si>
+    <t>Montenegro</t>
+  </si>
+  <si>
+    <t>Morocco</t>
+  </si>
+  <si>
+    <t>Mozambique</t>
+  </si>
+  <si>
+    <t>Myanmar</t>
+  </si>
+  <si>
+    <t>Namibia</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Nicaragua</t>
+  </si>
+  <si>
+    <t>Niger</t>
+  </si>
+  <si>
+    <t>Nigeria</t>
+  </si>
+  <si>
+    <t>North Korea</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>Nepal</t>
+  </si>
+  <si>
+    <t>New Zealand</t>
+  </si>
+  <si>
+    <t>Oman</t>
+  </si>
+  <si>
+    <t>Pakistan</t>
+  </si>
+  <si>
+    <t>Palestine</t>
+  </si>
+  <si>
+    <t>Palau</t>
+  </si>
+  <si>
+    <t>Panama</t>
+  </si>
+  <si>
+    <t>Papua New Guinea</t>
+  </si>
+  <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t>Philippines</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Romania</t>
+  </si>
+  <si>
+    <t>Russia</t>
+  </si>
+  <si>
+    <t>Rwanda</t>
+  </si>
+  <si>
+    <t>South Africa</t>
+  </si>
+  <si>
+    <t>Samoa</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>Senegal</t>
+  </si>
+  <si>
+    <t>Serbia</t>
+  </si>
+  <si>
+    <t>Seychelles</t>
+  </si>
+  <si>
+    <t>Thailand</t>
+  </si>
+  <si>
+    <t>St. Kitts and Nevis</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>Sierra Leone</t>
+  </si>
+  <si>
+    <t>Slovakia</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>St. Lucia</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Solomon Islands</t>
+  </si>
+  <si>
+    <t>Somalia</t>
+  </si>
+  <si>
+    <t>Somaliland</t>
+  </si>
+  <si>
+    <t>South Ossetia</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Sri Lanka</t>
+  </si>
+  <si>
+    <t>South Sudan</t>
+  </si>
+  <si>
+    <t>São Tomé and Príncipe</t>
+  </si>
+  <si>
+    <t>Sudan</t>
+  </si>
+  <si>
+    <t>Suriname</t>
+  </si>
+  <si>
+    <t>St. Vincent and the Grenadines</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Syria</t>
+  </si>
+  <si>
+    <t>Republic of China</t>
+  </si>
+  <si>
+    <t>Tajikistan</t>
+  </si>
+  <si>
+    <t>Tanzania</t>
+  </si>
+  <si>
+    <t>Togo</t>
+  </si>
+  <si>
+    <t>Tonga</t>
+  </si>
+  <si>
+    <t>Transnistria</t>
+  </si>
+  <si>
+    <t>Trinidad and Tobago</t>
+  </si>
+  <si>
+    <t>Turkmenistan</t>
+  </si>
+  <si>
+    <t>Tunisia</t>
+  </si>
+  <si>
+    <t>Türkiye</t>
+  </si>
+  <si>
+    <t>Tuvalu</t>
+  </si>
+  <si>
+    <t>United Arab Emirates</t>
+  </si>
+  <si>
+    <t>Uganda</t>
+  </si>
+  <si>
+    <t>Ukraine</t>
+  </si>
+  <si>
+    <t>Uruguay</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Uzbekistan</t>
+  </si>
+  <si>
+    <t>Vanuatu</t>
+  </si>
+  <si>
+    <t>Venezuela</t>
+  </si>
+  <si>
+    <t>Vietnam</t>
+  </si>
+  <si>
+    <t>Yemen</t>
+  </si>
+  <si>
+    <t>Zambia</t>
+  </si>
+  <si>
+    <t>Zimbabwe</t>
   </si>
 </sst>
 </file>
@@ -810,7 +1383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -824,6 +1397,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1161,8 +1735,8 @@
   <dimension ref="A1:L203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
@@ -1212,7 +1786,7 @@
       <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="13" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -1281,1159 +1855,1923 @@
       <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
+      <c r="B11" s="1" t="s">
+        <v>231</v>
+      </c>
       <c r="D11" s="2"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="B12" s="1" t="s">
+        <v>216</v>
+      </c>
       <c r="D12" s="2"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>23</v>
       </c>
+      <c r="B13" s="1" t="s">
+        <v>234</v>
+      </c>
       <c r="D13" s="2"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>24</v>
       </c>
+      <c r="B14" s="1" t="s">
+        <v>217</v>
+      </c>
       <c r="D14" s="2"/>
+      <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>25</v>
       </c>
+      <c r="B15" s="1" t="s">
+        <v>218</v>
+      </c>
       <c r="D15" s="2"/>
+      <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>26</v>
       </c>
+      <c r="B16" s="1" t="s">
+        <v>219</v>
+      </c>
       <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>27</v>
       </c>
+      <c r="B17" s="1" t="s">
+        <v>220</v>
+      </c>
       <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>28</v>
       </c>
+      <c r="B18" s="1" t="s">
+        <v>221</v>
+      </c>
       <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>29</v>
       </c>
+      <c r="B19" s="1" t="s">
+        <v>222</v>
+      </c>
       <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="B20" s="1" t="s">
+        <v>223</v>
+      </c>
       <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
+      <c r="B21" s="1" t="s">
+        <v>224</v>
+      </c>
       <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>32</v>
       </c>
+      <c r="B22" s="1" t="s">
+        <v>233</v>
+      </c>
       <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>33</v>
       </c>
+      <c r="B23" s="1" t="s">
+        <v>225</v>
+      </c>
       <c r="D23" s="2"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>34</v>
       </c>
+      <c r="B24" s="1" t="s">
+        <v>226</v>
+      </c>
       <c r="D24" s="2"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>35</v>
       </c>
+      <c r="B25" s="1" t="s">
+        <v>227</v>
+      </c>
       <c r="D25" s="2"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>36</v>
       </c>
+      <c r="B26" s="1" t="s">
+        <v>228</v>
+      </c>
       <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>37</v>
       </c>
+      <c r="B27" s="1" t="s">
+        <v>229</v>
+      </c>
       <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>38</v>
       </c>
+      <c r="B28" s="1" t="s">
+        <v>230</v>
+      </c>
       <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>39</v>
       </c>
+      <c r="B29" s="1" t="s">
+        <v>232</v>
+      </c>
       <c r="D29" s="2"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>40</v>
       </c>
+      <c r="B30" s="1" t="s">
+        <v>235</v>
+      </c>
       <c r="D30" s="2"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>41</v>
       </c>
+      <c r="B31" s="1" t="s">
+        <v>236</v>
+      </c>
       <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>2</v>
       </c>
+      <c r="B32" s="1" t="s">
+        <v>237</v>
+      </c>
       <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>42</v>
       </c>
+      <c r="B33" s="1" t="s">
+        <v>238</v>
+      </c>
       <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>43</v>
       </c>
+      <c r="B34" s="1" t="s">
+        <v>239</v>
+      </c>
       <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="B35" s="1" t="s">
+        <v>240</v>
+      </c>
       <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>45</v>
       </c>
+      <c r="B36" s="1" t="s">
+        <v>241</v>
+      </c>
       <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36" s="3"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>46</v>
       </c>
+      <c r="B37" s="1" t="s">
+        <v>242</v>
+      </c>
       <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>47</v>
       </c>
+      <c r="B38" s="1" t="s">
+        <v>243</v>
+      </c>
       <c r="D38" s="2"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>48</v>
       </c>
+      <c r="B39" s="1" t="s">
+        <v>244</v>
+      </c>
       <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>49</v>
       </c>
+      <c r="B40" s="1" t="s">
+        <v>245</v>
+      </c>
       <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>50</v>
       </c>
+      <c r="B41" s="1" t="s">
+        <v>246</v>
+      </c>
       <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>51</v>
       </c>
+      <c r="B42" s="1" t="s">
+        <v>247</v>
+      </c>
       <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E42" s="3"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>52</v>
       </c>
+      <c r="B43" s="1" t="s">
+        <v>249</v>
+      </c>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>53</v>
       </c>
+      <c r="B44" s="1" t="s">
+        <v>248</v>
+      </c>
       <c r="D44" s="2"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E44" s="3"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>54</v>
       </c>
+      <c r="B45" s="1" t="s">
+        <v>250</v>
+      </c>
       <c r="D45" s="2"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45" s="3"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>55</v>
       </c>
+      <c r="B46" s="1" t="s">
+        <v>251</v>
+      </c>
       <c r="D46" s="2"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46" s="3"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>56</v>
       </c>
+      <c r="B47" s="1" t="s">
+        <v>252</v>
+      </c>
       <c r="D47" s="2"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47" s="3"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>57</v>
       </c>
+      <c r="B48" s="1" t="s">
+        <v>253</v>
+      </c>
       <c r="D48" s="2"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E48" s="3"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>58</v>
       </c>
+      <c r="B49" s="1" t="s">
+        <v>254</v>
+      </c>
       <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" s="3"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>59</v>
       </c>
+      <c r="B50" s="1" t="s">
+        <v>255</v>
+      </c>
       <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E50" s="3"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>60</v>
       </c>
+      <c r="B51" s="1" t="s">
+        <v>256</v>
+      </c>
       <c r="D51" s="2"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" s="3"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>61</v>
       </c>
+      <c r="B52" s="1" t="s">
+        <v>257</v>
+      </c>
       <c r="D52" s="2"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" s="3"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>62</v>
       </c>
+      <c r="B53" s="1" t="s">
+        <v>258</v>
+      </c>
       <c r="D53" s="2"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" s="3"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>63</v>
       </c>
+      <c r="B54" s="1" t="s">
+        <v>259</v>
+      </c>
       <c r="D54" s="2"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E54" s="3"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>64</v>
       </c>
       <c r="D55" s="2"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>65</v>
       </c>
+      <c r="B56" s="1" t="s">
+        <v>260</v>
+      </c>
       <c r="D56" s="2"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E56" s="3"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>66</v>
       </c>
+      <c r="B57" s="1" t="s">
+        <v>261</v>
+      </c>
       <c r="D57" s="2"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E57" s="3"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="B58" s="1" t="s">
+        <v>262</v>
+      </c>
       <c r="D58" s="2"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="B59" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="D59" s="2"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E59" s="3"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>69</v>
       </c>
+      <c r="B60" s="1" t="s">
+        <v>264</v>
+      </c>
       <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E60" s="3"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>70</v>
       </c>
+      <c r="B61" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="D61" s="2"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E61" s="3"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>71</v>
       </c>
+      <c r="B62" s="1" t="s">
+        <v>266</v>
+      </c>
       <c r="D62" s="2"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E62" s="3"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>72</v>
       </c>
+      <c r="B63" s="1" t="s">
+        <v>267</v>
+      </c>
       <c r="D63" s="2"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>74</v>
       </c>
+      <c r="B64" s="1" t="s">
+        <v>268</v>
+      </c>
       <c r="D64" s="2"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>73</v>
       </c>
+      <c r="B65" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E65" s="3"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>75</v>
       </c>
+      <c r="B66" s="1" t="s">
+        <v>270</v>
+      </c>
       <c r="D66" s="2"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E66" s="3"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>76</v>
       </c>
+      <c r="B67" s="1" t="s">
+        <v>271</v>
+      </c>
       <c r="D67" s="2"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E67" s="3"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>77</v>
       </c>
+      <c r="B68" s="1" t="s">
+        <v>272</v>
+      </c>
       <c r="D68" s="2"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E68" s="3"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>78</v>
       </c>
+      <c r="B69" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E69" s="3"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>79</v>
       </c>
+      <c r="B70" s="1" t="s">
+        <v>274</v>
+      </c>
       <c r="D70" s="2"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E70" s="3"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>80</v>
       </c>
+      <c r="B71" s="1" t="s">
+        <v>275</v>
+      </c>
       <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71" s="3"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>81</v>
       </c>
+      <c r="B72" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="D72" s="2"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" s="3"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>1</v>
       </c>
+      <c r="B73" s="1" t="s">
+        <v>277</v>
+      </c>
       <c r="D73" s="2"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E73" s="3"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>82</v>
       </c>
+      <c r="B74" s="1" t="s">
+        <v>278</v>
+      </c>
       <c r="D74" s="2"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E74" s="3"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>83</v>
       </c>
+      <c r="B75" s="1" t="s">
+        <v>279</v>
+      </c>
       <c r="D75" s="2"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E75" s="3"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
         <v>84</v>
       </c>
+      <c r="B76" s="1" t="s">
+        <v>280</v>
+      </c>
       <c r="D76" s="2"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" s="3"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>85</v>
       </c>
+      <c r="B77" s="1" t="s">
+        <v>281</v>
+      </c>
       <c r="D77" s="2"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E77" s="3"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
         <v>86</v>
       </c>
+      <c r="B78" s="1" t="s">
+        <v>282</v>
+      </c>
       <c r="D78" s="2"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E78" s="3"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>87</v>
       </c>
+      <c r="B79" s="1" t="s">
+        <v>283</v>
+      </c>
       <c r="D79" s="2"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E79" s="3"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
         <v>88</v>
       </c>
+      <c r="B80" s="1" t="s">
+        <v>284</v>
+      </c>
       <c r="D80" s="2"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E80" s="3"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>89</v>
       </c>
+      <c r="B81" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="D81" s="2"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E81" s="3"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
         <v>90</v>
       </c>
+      <c r="B82" s="1" t="s">
+        <v>286</v>
+      </c>
       <c r="D82" s="2"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E82" s="3"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>91</v>
       </c>
+      <c r="B83" s="1" t="s">
+        <v>287</v>
+      </c>
       <c r="D83" s="2"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E83" s="3"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
         <v>92</v>
       </c>
+      <c r="B84" s="1" t="s">
+        <v>288</v>
+      </c>
       <c r="D84" s="2"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E84" s="3"/>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>93</v>
       </c>
+      <c r="B85" s="1" t="s">
+        <v>289</v>
+      </c>
       <c r="D85" s="2"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E85" s="3"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
         <v>94</v>
       </c>
+      <c r="B86" s="1" t="s">
+        <v>290</v>
+      </c>
       <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E86" s="3"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>95</v>
       </c>
+      <c r="B87" s="1" t="s">
+        <v>291</v>
+      </c>
       <c r="D87" s="2"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E87" s="3"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
         <v>96</v>
       </c>
+      <c r="B88" s="1" t="s">
+        <v>292</v>
+      </c>
       <c r="D88" s="2"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E88" s="3"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>97</v>
       </c>
+      <c r="B89" s="1" t="s">
+        <v>293</v>
+      </c>
       <c r="D89" s="2"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E89" s="3"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
         <v>98</v>
       </c>
+      <c r="B90" s="1" t="s">
+        <v>294</v>
+      </c>
       <c r="D90" s="2"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E90" s="3"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>99</v>
       </c>
+      <c r="B91" s="1" t="s">
+        <v>295</v>
+      </c>
       <c r="D91" s="2"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E91" s="3"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
         <v>100</v>
       </c>
+      <c r="B92" s="1" t="s">
+        <v>296</v>
+      </c>
       <c r="D92" s="2"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E92" s="3"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>101</v>
       </c>
+      <c r="B93" s="1" t="s">
+        <v>297</v>
+      </c>
       <c r="D93" s="2"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" s="3"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>102</v>
       </c>
+      <c r="B94" s="1" t="s">
+        <v>298</v>
+      </c>
       <c r="D94" s="2"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" s="3"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>103</v>
       </c>
+      <c r="B95" s="1" t="s">
+        <v>299</v>
+      </c>
       <c r="D95" s="2"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E95" s="3"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>104</v>
       </c>
+      <c r="B96" s="1" t="s">
+        <v>300</v>
+      </c>
       <c r="D96" s="2"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E96" s="3"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
         <v>105</v>
       </c>
+      <c r="B97" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="D97" s="2"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" s="3"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
         <v>106</v>
       </c>
+      <c r="B98" s="1" t="s">
+        <v>302</v>
+      </c>
       <c r="D98" s="2"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" s="3"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>109</v>
       </c>
+      <c r="B99" s="1" t="s">
+        <v>303</v>
+      </c>
       <c r="D99" s="2"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" s="3"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
         <v>3</v>
       </c>
+      <c r="B100" s="1" t="s">
+        <v>304</v>
+      </c>
       <c r="D100" s="2"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" s="3"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
         <v>107</v>
       </c>
+      <c r="B101" s="1" t="s">
+        <v>305</v>
+      </c>
       <c r="D101" s="2"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E101" s="3"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
         <v>108</v>
       </c>
+      <c r="B102" s="1" t="s">
+        <v>306</v>
+      </c>
       <c r="D102" s="2"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E102" s="3"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
         <v>110</v>
       </c>
+      <c r="B103" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="D103" s="2"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E103" s="3"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
         <v>111</v>
       </c>
+      <c r="B104" s="1" t="s">
+        <v>308</v>
+      </c>
       <c r="D104" s="2"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E104" s="3"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>112</v>
       </c>
+      <c r="B105" s="1" t="s">
+        <v>309</v>
+      </c>
       <c r="D105" s="2"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E105" s="3"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>113</v>
       </c>
+      <c r="B106" s="1" t="s">
+        <v>310</v>
+      </c>
       <c r="D106" s="2"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E106" s="3"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
         <v>114</v>
       </c>
+      <c r="B107" s="1" t="s">
+        <v>311</v>
+      </c>
       <c r="D107" s="2"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E107" s="3"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="7" t="s">
         <v>115</v>
       </c>
+      <c r="B108" s="1" t="s">
+        <v>312</v>
+      </c>
       <c r="D108" s="2"/>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E108" s="3"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
         <v>116</v>
       </c>
+      <c r="B109" s="1" t="s">
+        <v>313</v>
+      </c>
       <c r="D109" s="2"/>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E109" s="3"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
         <v>117</v>
       </c>
+      <c r="B110" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="D110" s="2"/>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E110" s="3"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
         <v>118</v>
       </c>
+      <c r="B111" s="1" t="s">
+        <v>315</v>
+      </c>
       <c r="D111" s="2"/>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E111" s="3"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="7" t="s">
         <v>119</v>
       </c>
+      <c r="B112" s="1" t="s">
+        <v>317</v>
+      </c>
       <c r="D112" s="2"/>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E112" s="3"/>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
         <v>120</v>
       </c>
+      <c r="B113" s="1" t="s">
+        <v>316</v>
+      </c>
       <c r="D113" s="2"/>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E113" s="3"/>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="7" t="s">
         <v>121</v>
       </c>
+      <c r="B114" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="D114" s="2"/>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E114" s="3"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>122</v>
       </c>
+      <c r="B115" s="1" t="s">
+        <v>319</v>
+      </c>
       <c r="D115" s="2"/>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E115" s="3"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="7" t="s">
         <v>123</v>
       </c>
+      <c r="B116" s="1" t="s">
+        <v>320</v>
+      </c>
       <c r="D116" s="2"/>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E116" s="3"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
         <v>124</v>
       </c>
+      <c r="B117" s="1" t="s">
+        <v>321</v>
+      </c>
       <c r="D117" s="2"/>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E117" s="3"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="7" t="s">
         <v>125</v>
       </c>
+      <c r="B118" s="1" t="s">
+        <v>322</v>
+      </c>
       <c r="D118" s="2"/>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E118" s="3"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>126</v>
       </c>
+      <c r="B119" s="1" t="s">
+        <v>323</v>
+      </c>
       <c r="D119" s="2"/>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E119" s="3"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="7" t="s">
         <v>127</v>
       </c>
+      <c r="B120" s="1" t="s">
+        <v>323</v>
+      </c>
       <c r="D120" s="2"/>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E120" s="3"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
         <v>128</v>
       </c>
+      <c r="B121" s="1" t="s">
+        <v>324</v>
+      </c>
       <c r="D121" s="2"/>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E121" s="3"/>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="7" t="s">
         <v>129</v>
       </c>
+      <c r="B122" s="1" t="s">
+        <v>325</v>
+      </c>
       <c r="D122" s="2"/>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E122" s="3"/>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
         <v>130</v>
       </c>
+      <c r="B123" s="1" t="s">
+        <v>327</v>
+      </c>
       <c r="D123" s="2"/>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="7" t="s">
         <v>131</v>
       </c>
+      <c r="B124" s="1" t="s">
+        <v>326</v>
+      </c>
       <c r="D124" s="2"/>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E124" s="3"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
         <v>132</v>
       </c>
+      <c r="B125" s="1" t="s">
+        <v>328</v>
+      </c>
       <c r="D125" s="2"/>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E125" s="3"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
         <v>133</v>
       </c>
+      <c r="B126" s="1" t="s">
+        <v>329</v>
+      </c>
       <c r="D126" s="2"/>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E126" s="3"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
         <v>134</v>
       </c>
+      <c r="B127" s="1" t="s">
+        <v>330</v>
+      </c>
       <c r="D127" s="2"/>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E127" s="3"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="7" t="s">
         <v>135</v>
       </c>
+      <c r="B128" s="1" t="s">
+        <v>331</v>
+      </c>
       <c r="D128" s="2"/>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E128" s="3"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>136</v>
       </c>
+      <c r="B129" s="1" t="s">
+        <v>332</v>
+      </c>
       <c r="D129" s="2"/>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E129" s="3"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="7" t="s">
         <v>137</v>
       </c>
+      <c r="B130" s="1" t="s">
+        <v>333</v>
+      </c>
       <c r="D130" s="2"/>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E130" s="3"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
         <v>138</v>
       </c>
+      <c r="B131" s="1" t="s">
+        <v>334</v>
+      </c>
       <c r="D131" s="2"/>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E131" s="3"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="7" t="s">
         <v>139</v>
       </c>
+      <c r="B132" s="1" t="s">
+        <v>335</v>
+      </c>
       <c r="D132" s="2"/>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E132" s="3"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
         <v>140</v>
       </c>
+      <c r="B133" s="1" t="s">
+        <v>336</v>
+      </c>
       <c r="D133" s="2"/>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E133" s="3"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>141</v>
       </c>
+      <c r="B134" s="1" t="s">
+        <v>337</v>
+      </c>
       <c r="D134" s="2"/>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E134" s="3"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>142</v>
       </c>
+      <c r="B135" s="1" t="s">
+        <v>338</v>
+      </c>
       <c r="D135" s="2"/>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E135" s="3"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>143</v>
       </c>
+      <c r="B136" s="1" t="s">
+        <v>339</v>
+      </c>
       <c r="D136" s="2"/>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E136" s="3"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
         <v>144</v>
       </c>
+      <c r="B137" s="1" t="s">
+        <v>340</v>
+      </c>
       <c r="D137" s="2"/>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E137" s="3"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>145</v>
       </c>
+      <c r="B138" s="1" t="s">
+        <v>341</v>
+      </c>
       <c r="D138" s="2"/>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E138" s="3"/>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>146</v>
       </c>
+      <c r="B139" t="s">
+        <v>342</v>
+      </c>
       <c r="D139" s="2"/>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E139" s="3"/>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
         <v>147</v>
       </c>
+      <c r="B140" s="1" t="s">
+        <v>343</v>
+      </c>
       <c r="D140" s="2"/>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E140" s="3"/>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>148</v>
       </c>
+      <c r="B141" s="1" t="s">
+        <v>344</v>
+      </c>
       <c r="D141" s="2"/>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E141" s="3"/>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="7" t="s">
         <v>149</v>
       </c>
+      <c r="B142" s="1" t="s">
+        <v>345</v>
+      </c>
       <c r="D142" s="2"/>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E142" s="3"/>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>150</v>
       </c>
+      <c r="B143" s="1" t="s">
+        <v>346</v>
+      </c>
       <c r="D143" s="2"/>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E143" s="3"/>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="7" t="s">
         <v>151</v>
       </c>
+      <c r="B144" s="1" t="s">
+        <v>347</v>
+      </c>
       <c r="D144" s="2"/>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E144" s="3"/>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>152</v>
       </c>
+      <c r="B145" s="1" t="s">
+        <v>348</v>
+      </c>
       <c r="D145" s="2"/>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E145" s="3"/>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>153</v>
       </c>
+      <c r="B146" s="1" t="s">
+        <v>349</v>
+      </c>
       <c r="D146" s="2"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>154</v>
       </c>
+      <c r="B147" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="D147" s="2"/>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E147" s="3"/>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
         <v>155</v>
       </c>
+      <c r="B148" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="D148" s="2"/>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E148" s="3"/>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
         <v>156</v>
       </c>
+      <c r="B149" s="1" t="s">
+        <v>352</v>
+      </c>
       <c r="D149" s="2"/>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E149" s="3"/>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
         <v>157</v>
       </c>
+      <c r="B150" s="1" t="s">
+        <v>353</v>
+      </c>
       <c r="D150" s="2"/>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E150" s="3"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>158</v>
       </c>
+      <c r="B151" s="1" t="s">
+        <v>354</v>
+      </c>
       <c r="D151" s="2"/>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E151" s="3"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="7" t="s">
         <v>159</v>
       </c>
+      <c r="B152" s="1" t="s">
+        <v>355</v>
+      </c>
       <c r="D152" s="2"/>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E152" s="3"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
         <v>160</v>
       </c>
+      <c r="B153" s="1" t="s">
+        <v>356</v>
+      </c>
       <c r="D153" s="2"/>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E153" s="3"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="7" t="s">
         <v>161</v>
       </c>
+      <c r="B154" s="1" t="s">
+        <v>357</v>
+      </c>
       <c r="D154" s="2"/>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E154" s="3"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
         <v>162</v>
       </c>
+      <c r="B155" s="1" t="s">
+        <v>358</v>
+      </c>
       <c r="D155" s="2"/>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E155" s="3"/>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="7" t="s">
         <v>163</v>
       </c>
+      <c r="B156" s="1" t="s">
+        <v>359</v>
+      </c>
       <c r="D156" s="2"/>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E156" s="3"/>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
         <v>164</v>
       </c>
+      <c r="B157" s="1" t="s">
+        <v>360</v>
+      </c>
       <c r="D157" s="2"/>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E157" s="3"/>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="7" t="s">
         <v>165</v>
       </c>
+      <c r="B158" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="D158" s="2"/>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E158" s="3"/>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
         <v>166</v>
       </c>
+      <c r="B159" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="D159" s="2"/>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E159" s="3"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>168</v>
       </c>
+      <c r="B160" s="1" t="s">
+        <v>363</v>
+      </c>
       <c r="D160" s="2"/>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E160" s="3"/>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
         <v>169</v>
       </c>
+      <c r="B161" s="1" t="s">
+        <v>364</v>
+      </c>
       <c r="D161" s="2"/>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E161" s="3"/>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="7" t="s">
         <v>170</v>
       </c>
+      <c r="B162" s="1" t="s">
+        <v>365</v>
+      </c>
       <c r="D162" s="2"/>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E162" s="3"/>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="7" t="s">
         <v>171</v>
       </c>
+      <c r="B163" s="1" t="s">
+        <v>366</v>
+      </c>
       <c r="D163" s="2"/>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E163" s="3"/>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="7" t="s">
         <v>172</v>
       </c>
+      <c r="B164" s="1" t="s">
+        <v>367</v>
+      </c>
       <c r="D164" s="2"/>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E164" s="3"/>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>173</v>
       </c>
+      <c r="B165" s="1" t="s">
+        <v>368</v>
+      </c>
       <c r="D165" s="2"/>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E165" s="3"/>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="7" t="s">
         <v>167</v>
       </c>
+      <c r="B166" s="1" t="s">
+        <v>369</v>
+      </c>
       <c r="D166" s="2"/>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E166" s="3"/>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>174</v>
       </c>
+      <c r="B167" s="1" t="s">
+        <v>370</v>
+      </c>
       <c r="D167" s="2"/>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E167" s="3"/>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="7" t="s">
         <v>175</v>
       </c>
+      <c r="B168" s="1" t="s">
+        <v>371</v>
+      </c>
       <c r="D168" s="2"/>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E168" s="3"/>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="7" t="s">
         <v>176</v>
       </c>
+      <c r="B169" s="1" t="s">
+        <v>372</v>
+      </c>
       <c r="D169" s="2"/>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E169" s="3"/>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="7" t="s">
         <v>177</v>
       </c>
+      <c r="B170" s="1" t="s">
+        <v>373</v>
+      </c>
       <c r="D170" s="2"/>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E170" s="3"/>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
         <v>178</v>
       </c>
+      <c r="B171" s="1" t="s">
+        <v>374</v>
+      </c>
       <c r="D171" s="2"/>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E171" s="3"/>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="7" t="s">
         <v>179</v>
       </c>
+      <c r="B172" s="1" t="s">
+        <v>375</v>
+      </c>
       <c r="D172" s="2"/>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E172" s="3"/>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="7" t="s">
         <v>180</v>
       </c>
+      <c r="B173" s="1" t="s">
+        <v>376</v>
+      </c>
       <c r="D173" s="2"/>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E173" s="3"/>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="7" t="s">
         <v>181</v>
       </c>
+      <c r="B174" s="1" t="s">
+        <v>377</v>
+      </c>
       <c r="D174" s="2"/>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E174" s="3"/>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="7" t="s">
         <v>182</v>
       </c>
+      <c r="B175" s="1" t="s">
+        <v>378</v>
+      </c>
       <c r="D175" s="2"/>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E175" s="3"/>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="7" t="s">
         <v>183</v>
       </c>
+      <c r="B176" s="1" t="s">
+        <v>379</v>
+      </c>
       <c r="D176" s="2"/>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E176" s="3"/>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
         <v>184</v>
       </c>
+      <c r="B177" s="1" t="s">
+        <v>380</v>
+      </c>
       <c r="D177" s="2"/>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E177" s="3"/>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="7" t="s">
         <v>185</v>
       </c>
+      <c r="B178" s="1" t="s">
+        <v>381</v>
+      </c>
       <c r="D178" s="2"/>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E178" s="3"/>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>0</v>
       </c>
+      <c r="B179" s="1" t="s">
+        <v>382</v>
+      </c>
       <c r="D179" s="2"/>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E179" s="3"/>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
         <v>186</v>
       </c>
+      <c r="B180" s="1" t="s">
+        <v>383</v>
+      </c>
       <c r="D180" s="2"/>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E180" s="3"/>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
         <v>187</v>
       </c>
+      <c r="B181" s="1" t="s">
+        <v>384</v>
+      </c>
       <c r="D181" s="2"/>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E181" s="3"/>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
         <v>188</v>
       </c>
+      <c r="B182" s="1" t="s">
+        <v>385</v>
+      </c>
       <c r="D182" s="2"/>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E182" s="3"/>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="7" t="s">
         <v>189</v>
       </c>
+      <c r="B183" s="1" t="s">
+        <v>386</v>
+      </c>
       <c r="D183" s="2"/>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E183" s="3"/>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="7" t="s">
         <v>190</v>
       </c>
+      <c r="B184" s="1" t="s">
+        <v>388</v>
+      </c>
       <c r="D184" s="2"/>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E184" s="3"/>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
         <v>191</v>
       </c>
+      <c r="B185" s="1" t="s">
+        <v>387</v>
+      </c>
       <c r="D185" s="2"/>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E185" s="3"/>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="7" t="s">
         <v>193</v>
       </c>
+      <c r="B186" s="1" t="s">
+        <v>389</v>
+      </c>
       <c r="D186" s="2"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
         <v>192</v>
       </c>
+      <c r="B187" s="1" t="s">
+        <v>390</v>
+      </c>
       <c r="D187" s="2"/>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E187" s="3"/>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
         <v>194</v>
       </c>
+      <c r="B188" s="1" t="s">
+        <v>391</v>
+      </c>
       <c r="D188" s="2"/>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E188" s="3"/>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="7" t="s">
         <v>195</v>
       </c>
+      <c r="B189" s="1" t="s">
+        <v>392</v>
+      </c>
       <c r="D189" s="2"/>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E189" s="3"/>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="7" t="s">
         <v>196</v>
       </c>
+      <c r="B190" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="D190" s="2"/>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E190" s="3"/>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="7" t="s">
         <v>197</v>
       </c>
+      <c r="B191" s="1" t="s">
+        <v>394</v>
+      </c>
       <c r="D191" s="2"/>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E191" s="3"/>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="7" t="s">
         <v>198</v>
       </c>
+      <c r="B192" s="1" t="s">
+        <v>395</v>
+      </c>
       <c r="D192" s="2"/>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E192" s="3"/>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="7" t="s">
         <v>199</v>
       </c>
+      <c r="B193" s="1" t="s">
+        <v>396</v>
+      </c>
       <c r="D193" s="2"/>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E193" s="3"/>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
         <v>200</v>
       </c>
+      <c r="B194" s="1" t="s">
+        <v>397</v>
+      </c>
       <c r="D194" s="2"/>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E194" s="3"/>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="7" t="s">
         <v>201</v>
       </c>
+      <c r="B195" s="1" t="s">
+        <v>398</v>
+      </c>
       <c r="D195" s="2"/>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E195" s="3"/>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="7" t="s">
         <v>202</v>
       </c>
+      <c r="B196" s="1" t="s">
+        <v>399</v>
+      </c>
       <c r="D196" s="2"/>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E196" s="3"/>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="7" t="s">
         <v>203</v>
       </c>
+      <c r="B197" s="1" t="s">
+        <v>400</v>
+      </c>
       <c r="D197" s="2"/>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E197" s="3"/>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
         <v>204</v>
       </c>
+      <c r="B198" s="1" t="s">
+        <v>401</v>
+      </c>
       <c r="D198" s="2"/>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E198" s="3"/>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>205</v>
       </c>
+      <c r="B199" s="1" t="s">
+        <v>402</v>
+      </c>
       <c r="D199" s="2"/>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E199" s="3"/>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="7" t="s">
         <v>206</v>
       </c>
+      <c r="B200" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="D200" s="2"/>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E200" s="3"/>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="7" t="s">
         <v>207</v>
       </c>
+      <c r="B201" s="1" t="s">
+        <v>404</v>
+      </c>
       <c r="D201" s="2"/>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E201" s="3"/>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
         <v>208</v>
       </c>
+      <c r="B202" s="1" t="s">
+        <v>405</v>
+      </c>
       <c r="D202" s="2"/>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E202" s="3"/>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
         <v>209</v>
       </c>
+      <c r="B203" s="1" t="s">
+        <v>406</v>
+      </c>
       <c r="D203" s="2"/>
+      <c r="E203" s="3"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A7:A203">

</xml_diff>

<commit_message>
Add two properties to progress table
</commit_message>
<xml_diff>
--- a/countries_progress.xlsx
+++ b/countries_progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Desktop\Modern-Day-Mod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE84AA3-5827-4FFF-B8F6-6B3DE038D532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65079E5-B736-45C4-846E-D1F4A09C993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25200" yWindow="0" windowWidth="12600" windowHeight="15300" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15540" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="409">
   <si>
     <t>SWI</t>
   </si>
@@ -1257,6 +1257,12 @@
   </si>
   <si>
     <t>Zimbabwe</t>
+  </si>
+  <si>
+    <t>Vegetation</t>
+  </si>
+  <si>
+    <t>RGOs/Goods</t>
   </si>
 </sst>
 </file>
@@ -1397,7 +1403,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1732,7 +1738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398DC3DE-D0FA-422E-8FF2-6EBA966CD369}">
-  <dimension ref="A1:L203"/>
+  <dimension ref="A1:N203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="7" bestFit="1" customWidth="1"/>
@@ -1748,36 +1754,36 @@
     <col min="12" max="12" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="8"/>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12"/>
       <c r="B6" s="5"/>
       <c r="C6" s="6" t="s">
@@ -1810,8 +1816,14 @@
       <c r="L6" s="6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>17</v>
       </c>
@@ -1821,7 +1833,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>18</v>
       </c>
@@ -1831,7 +1843,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>19</v>
       </c>
@@ -1841,7 +1853,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
@@ -1851,7 +1863,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
@@ -1861,7 +1873,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
@@ -1871,7 +1883,7 @@
       <c r="D12" s="2"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>23</v>
       </c>
@@ -1881,7 +1893,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>24</v>
       </c>
@@ -1891,7 +1903,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>25</v>
       </c>
@@ -1901,7 +1913,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
changed status of UK and ireland vegetation (provisionaly done)
</commit_message>
<xml_diff>
--- a/countries_progress.xlsx
+++ b/countries_progress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Desktop\Modern-Day-Mod\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karl\Documents\GitHub\Modern-Day-Mod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65079E5-B736-45C4-846E-D1F4A09C993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830AF526-4990-4186-9DCC-6BAADF42C0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15540" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1389,7 +1389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1403,10 +1403,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1739,7 +1738,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398DC3DE-D0FA-422E-8FF2-6EBA966CD369}">
   <dimension ref="A1:N203"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="1" bestFit="1" customWidth="1"/>
@@ -1792,7 +1791,7 @@
       <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -2398,7 +2397,7 @@
       <c r="D64" s="2"/>
       <c r="E64" s="3"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>73</v>
       </c>
@@ -2408,7 +2407,7 @@
       <c r="D65" s="2"/>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>75</v>
       </c>
@@ -2418,7 +2417,7 @@
       <c r="D66" s="2"/>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>76</v>
       </c>
@@ -2428,7 +2427,7 @@
       <c r="D67" s="2"/>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>77</v>
       </c>
@@ -2438,7 +2437,7 @@
       <c r="D68" s="2"/>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>78</v>
       </c>
@@ -2448,7 +2447,7 @@
       <c r="D69" s="2"/>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>79</v>
       </c>
@@ -2458,7 +2457,7 @@
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>80</v>
       </c>
@@ -2468,7 +2467,7 @@
       <c r="D71" s="2"/>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>81</v>
       </c>
@@ -2477,8 +2476,9 @@
       </c>
       <c r="D72" s="2"/>
       <c r="E72" s="3"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="M72" s="2"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>1</v>
       </c>
@@ -2488,7 +2488,7 @@
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>82</v>
       </c>
@@ -2498,7 +2498,7 @@
       <c r="D74" s="2"/>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>83</v>
       </c>
@@ -2508,7 +2508,7 @@
       <c r="D75" s="2"/>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
         <v>84</v>
       </c>
@@ -2518,7 +2518,7 @@
       <c r="D76" s="2"/>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>85</v>
       </c>
@@ -2528,7 +2528,7 @@
       <c r="D77" s="2"/>
       <c r="E77" s="3"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
         <v>86</v>
       </c>
@@ -2538,7 +2538,7 @@
       <c r="D78" s="2"/>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>87</v>
       </c>
@@ -2548,7 +2548,7 @@
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
         <v>88</v>
       </c>
@@ -2558,7 +2558,7 @@
       <c r="D80" s="2"/>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>89</v>
       </c>
@@ -2568,7 +2568,7 @@
       <c r="D81" s="2"/>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
         <v>90</v>
       </c>
@@ -2578,7 +2578,7 @@
       <c r="D82" s="2"/>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>91</v>
       </c>
@@ -2588,7 +2588,7 @@
       <c r="D83" s="2"/>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
         <v>92</v>
       </c>
@@ -2598,7 +2598,7 @@
       <c r="D84" s="2"/>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>93</v>
       </c>
@@ -2608,7 +2608,7 @@
       <c r="D85" s="2"/>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
         <v>94</v>
       </c>
@@ -2618,7 +2618,7 @@
       <c r="D86" s="2"/>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>95</v>
       </c>
@@ -2628,7 +2628,7 @@
       <c r="D87" s="2"/>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
         <v>96</v>
       </c>
@@ -2638,7 +2638,7 @@
       <c r="D88" s="2"/>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>97</v>
       </c>
@@ -2648,7 +2648,7 @@
       <c r="D89" s="2"/>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
         <v>98</v>
       </c>
@@ -2657,8 +2657,9 @@
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="M90" s="2"/>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>99</v>
       </c>
@@ -2668,7 +2669,7 @@
       <c r="D91" s="2"/>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
         <v>100</v>
       </c>
@@ -2678,7 +2679,7 @@
       <c r="D92" s="2"/>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>101</v>
       </c>
@@ -2688,7 +2689,7 @@
       <c r="D93" s="2"/>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>102</v>
       </c>
@@ -2698,7 +2699,7 @@
       <c r="D94" s="2"/>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>103</v>
       </c>
@@ -2708,7 +2709,7 @@
       <c r="D95" s="2"/>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>104</v>
       </c>

</xml_diff>

<commit_message>
Add flag of MICR (Micronesia)
</commit_message>
<xml_diff>
--- a/countries_progress.xlsx
+++ b/countries_progress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karl\Documents\GitHub\Modern-Day-Mod\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Desktop\Modern-Day-Mod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830AF526-4990-4186-9DCC-6BAADF42C0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A8ACF7-4057-40E5-A041-084CFE592634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15540" xr2:uid="{C597D0B7-6BAE-4019-B376-05F9FD1F1825}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -1405,7 +1405,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1738,7 +1738,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{398DC3DE-D0FA-422E-8FF2-6EBA966CD369}">
   <dimension ref="A1:N203"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="1" bestFit="1" customWidth="1"/>
@@ -2987,6 +2987,7 @@
         <v>327</v>
       </c>
       <c r="D123" s="2"/>
+      <c r="E123" s="3"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="7" t="s">

</xml_diff>